<commit_message>
Update generated outputs and config for all scenarios
</commit_message>
<xml_diff>
--- a/t1_confection/A1_Outputs/A1_Outputs_NDC/A-O_Demand.xlsx
+++ b/t1_confection/A1_Outputs/A1_Outputs_NDC/A-O_Demand.xlsx
@@ -738,88 +738,88 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>469.23</v>
+        <v>524.49</v>
       </c>
       <c r="J2" t="n">
-        <v>473.36</v>
+        <v>506.39</v>
       </c>
       <c r="K2" t="n">
-        <v>479.88</v>
+        <v>512</v>
       </c>
       <c r="L2" t="n">
-        <v>486.43</v>
+        <v>518.55</v>
       </c>
       <c r="M2" t="n">
-        <v>493.03</v>
+        <v>525.15</v>
       </c>
       <c r="N2" t="n">
-        <v>499.67</v>
+        <v>531.79</v>
       </c>
       <c r="O2" t="n">
-        <v>506.36</v>
+        <v>538.48</v>
       </c>
       <c r="P2" t="n">
-        <v>513.08</v>
+        <v>545.2</v>
       </c>
       <c r="Q2" t="n">
-        <v>519.84</v>
+        <v>551.96</v>
       </c>
       <c r="R2" t="n">
-        <v>526.65</v>
+        <v>558.77</v>
       </c>
       <c r="S2" t="n">
-        <v>533.5</v>
+        <v>565.62</v>
       </c>
       <c r="T2" t="n">
-        <v>540.38</v>
+        <v>572.5</v>
       </c>
       <c r="U2" t="n">
-        <v>547.3099999999999</v>
+        <v>579.4299999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>554.28</v>
+        <v>586.4</v>
       </c>
       <c r="W2" t="n">
-        <v>561.3</v>
+        <v>593.42</v>
       </c>
       <c r="X2" t="n">
-        <v>568.35</v>
+        <v>600.47</v>
       </c>
       <c r="Y2" t="n">
-        <v>575.45</v>
+        <v>607.5700000000001</v>
       </c>
       <c r="Z2" t="n">
-        <v>582.58</v>
+        <v>614.7</v>
       </c>
       <c r="AA2" t="n">
-        <v>589.76</v>
+        <v>621.88</v>
       </c>
       <c r="AB2" t="n">
-        <v>596.98</v>
+        <v>629.1</v>
       </c>
       <c r="AC2" t="n">
-        <v>604.24</v>
+        <v>636.36</v>
       </c>
       <c r="AD2" t="n">
-        <v>611.54</v>
+        <v>643.66</v>
       </c>
       <c r="AE2" t="n">
-        <v>618.88</v>
+        <v>651</v>
       </c>
       <c r="AF2" t="n">
-        <v>626.26</v>
+        <v>658.38</v>
       </c>
       <c r="AG2" t="n">
-        <v>633.6900000000001</v>
+        <v>665.8099999999999</v>
       </c>
       <c r="AH2" t="n">
-        <v>641.16</v>
+        <v>673.28</v>
       </c>
       <c r="AI2" t="n">
-        <v>648.66</v>
+        <v>680.78</v>
       </c>
       <c r="AJ2" t="n">
-        <v>656.21</v>
+        <v>688.33</v>
       </c>
     </row>
     <row r="3">
@@ -862,88 +862,88 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>43.08</v>
+        <v>42.81</v>
       </c>
       <c r="J3" t="n">
-        <v>45.83</v>
+        <v>45.15</v>
       </c>
       <c r="K3" t="n">
-        <v>48.82</v>
+        <v>48.63</v>
       </c>
       <c r="L3" t="n">
-        <v>51.84</v>
+        <v>51.65</v>
       </c>
       <c r="M3" t="n">
-        <v>54.88</v>
+        <v>54.69</v>
       </c>
       <c r="N3" t="n">
-        <v>57.96</v>
+        <v>57.77</v>
       </c>
       <c r="O3" t="n">
-        <v>61.06</v>
+        <v>60.87</v>
       </c>
       <c r="P3" t="n">
-        <v>64.19</v>
+        <v>64</v>
       </c>
       <c r="Q3" t="n">
-        <v>67.34</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="R3" t="n">
-        <v>70.53</v>
+        <v>70.34</v>
       </c>
       <c r="S3" t="n">
-        <v>73.73999999999999</v>
+        <v>73.55</v>
       </c>
       <c r="T3" t="n">
-        <v>76.98</v>
+        <v>76.79000000000001</v>
       </c>
       <c r="U3" t="n">
-        <v>80.23999999999999</v>
+        <v>80.05</v>
       </c>
       <c r="V3" t="n">
-        <v>83.54000000000001</v>
+        <v>83.34999999999999</v>
       </c>
       <c r="W3" t="n">
-        <v>86.86</v>
+        <v>86.67</v>
       </c>
       <c r="X3" t="n">
-        <v>90.20999999999999</v>
+        <v>90.02</v>
       </c>
       <c r="Y3" t="n">
-        <v>93.58</v>
+        <v>93.39</v>
       </c>
       <c r="Z3" t="n">
-        <v>96.98999999999999</v>
+        <v>96.8</v>
       </c>
       <c r="AA3" t="n">
-        <v>100.42</v>
+        <v>100.23</v>
       </c>
       <c r="AB3" t="n">
-        <v>103.88</v>
+        <v>103.69</v>
       </c>
       <c r="AC3" t="n">
-        <v>107.36</v>
+        <v>107.17</v>
       </c>
       <c r="AD3" t="n">
-        <v>110.88</v>
+        <v>110.69</v>
       </c>
       <c r="AE3" t="n">
-        <v>114.42</v>
+        <v>114.23</v>
       </c>
       <c r="AF3" t="n">
-        <v>117.99</v>
+        <v>117.8</v>
       </c>
       <c r="AG3" t="n">
-        <v>121.58</v>
+        <v>121.39</v>
       </c>
       <c r="AH3" t="n">
-        <v>125.21</v>
+        <v>125.02</v>
       </c>
       <c r="AI3" t="n">
-        <v>128.86</v>
+        <v>128.67</v>
       </c>
       <c r="AJ3" t="n">
-        <v>132.54</v>
+        <v>132.35</v>
       </c>
     </row>
     <row r="4">
@@ -986,88 +986,88 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>2549.23</v>
+        <v>2599.63</v>
       </c>
       <c r="J4" t="n">
-        <v>2605.06</v>
+        <v>2637.58</v>
       </c>
       <c r="K4" t="n">
-        <v>2674.19</v>
+        <v>2732.79</v>
       </c>
       <c r="L4" t="n">
-        <v>2743.88</v>
+        <v>2802.48</v>
       </c>
       <c r="M4" t="n">
-        <v>2814.13</v>
+        <v>2872.73</v>
       </c>
       <c r="N4" t="n">
-        <v>2884.94</v>
+        <v>2943.54</v>
       </c>
       <c r="O4" t="n">
-        <v>2956.3</v>
+        <v>3014.9</v>
       </c>
       <c r="P4" t="n">
-        <v>3028.23</v>
+        <v>3086.83</v>
       </c>
       <c r="Q4" t="n">
-        <v>3100.71</v>
+        <v>3159.31</v>
       </c>
       <c r="R4" t="n">
-        <v>3173.75</v>
+        <v>3232.35</v>
       </c>
       <c r="S4" t="n">
-        <v>3247.35</v>
+        <v>3305.95</v>
       </c>
       <c r="T4" t="n">
-        <v>3321.51</v>
+        <v>3380.11</v>
       </c>
       <c r="U4" t="n">
-        <v>3396.22</v>
+        <v>3454.82</v>
       </c>
       <c r="V4" t="n">
-        <v>3471.49</v>
+        <v>3530.09</v>
       </c>
       <c r="W4" t="n">
-        <v>3547.33</v>
+        <v>3605.93</v>
       </c>
       <c r="X4" t="n">
-        <v>3623.72</v>
+        <v>3682.32</v>
       </c>
       <c r="Y4" t="n">
-        <v>3700.66</v>
+        <v>3759.26</v>
       </c>
       <c r="Z4" t="n">
-        <v>3778.17</v>
+        <v>3836.77</v>
       </c>
       <c r="AA4" t="n">
-        <v>3856.24</v>
+        <v>3914.84</v>
       </c>
       <c r="AB4" t="n">
-        <v>3934.86</v>
+        <v>3993.46</v>
       </c>
       <c r="AC4" t="n">
-        <v>4014.04</v>
+        <v>4072.64</v>
       </c>
       <c r="AD4" t="n">
-        <v>4093.78</v>
+        <v>4152.38</v>
       </c>
       <c r="AE4" t="n">
-        <v>4174.08</v>
+        <v>4232.68</v>
       </c>
       <c r="AF4" t="n">
-        <v>4254.94</v>
+        <v>4313.54</v>
       </c>
       <c r="AG4" t="n">
-        <v>4336.35</v>
+        <v>4394.95</v>
       </c>
       <c r="AH4" t="n">
-        <v>4418.32</v>
+        <v>4476.92</v>
       </c>
       <c r="AI4" t="n">
-        <v>4500.86</v>
+        <v>4559.46</v>
       </c>
       <c r="AJ4" t="n">
-        <v>4583.94</v>
+        <v>4642.54</v>
       </c>
     </row>
     <row r="5">
@@ -1234,88 +1234,88 @@
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>302.39</v>
+        <v>302.25</v>
       </c>
       <c r="J6" t="n">
         <v>318.54</v>
       </c>
       <c r="K6" t="n">
-        <v>336.36</v>
+        <v>336.33</v>
       </c>
       <c r="L6" t="n">
-        <v>354.34</v>
+        <v>354.31</v>
       </c>
       <c r="M6" t="n">
-        <v>372.49</v>
+        <v>372.46</v>
       </c>
       <c r="N6" t="n">
-        <v>390.79</v>
+        <v>390.76</v>
       </c>
       <c r="O6" t="n">
-        <v>409.26</v>
+        <v>409.23</v>
       </c>
       <c r="P6" t="n">
-        <v>427.89</v>
+        <v>427.86</v>
       </c>
       <c r="Q6" t="n">
-        <v>446.68</v>
+        <v>446.65</v>
       </c>
       <c r="R6" t="n">
-        <v>465.63</v>
+        <v>465.6</v>
       </c>
       <c r="S6" t="n">
-        <v>484.74</v>
+        <v>484.71</v>
       </c>
       <c r="T6" t="n">
-        <v>504.02</v>
+        <v>503.99</v>
       </c>
       <c r="U6" t="n">
-        <v>523.46</v>
+        <v>523.4299999999999</v>
       </c>
       <c r="V6" t="n">
-        <v>543.05</v>
+        <v>543.02</v>
       </c>
       <c r="W6" t="n">
-        <v>562.8099999999999</v>
+        <v>562.78</v>
       </c>
       <c r="X6" t="n">
-        <v>582.73</v>
+        <v>582.7</v>
       </c>
       <c r="Y6" t="n">
-        <v>602.8099999999999</v>
+        <v>602.78</v>
       </c>
       <c r="Z6" t="n">
-        <v>623.0599999999999</v>
+        <v>623.03</v>
       </c>
       <c r="AA6" t="n">
-        <v>643.46</v>
+        <v>643.4299999999999</v>
       </c>
       <c r="AB6" t="n">
-        <v>664.03</v>
+        <v>664</v>
       </c>
       <c r="AC6" t="n">
-        <v>684.76</v>
+        <v>684.73</v>
       </c>
       <c r="AD6" t="n">
-        <v>705.65</v>
+        <v>705.62</v>
       </c>
       <c r="AE6" t="n">
-        <v>726.7</v>
+        <v>726.67</v>
       </c>
       <c r="AF6" t="n">
-        <v>747.91</v>
+        <v>747.88</v>
       </c>
       <c r="AG6" t="n">
-        <v>769.28</v>
+        <v>769.25</v>
       </c>
       <c r="AH6" t="n">
-        <v>790.8200000000001</v>
+        <v>790.79</v>
       </c>
       <c r="AI6" t="n">
-        <v>812.51</v>
+        <v>812.48</v>
       </c>
       <c r="AJ6" t="n">
-        <v>834.37</v>
+        <v>834.34</v>
       </c>
     </row>
     <row r="7">
@@ -1358,88 +1358,88 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>290.09</v>
+        <v>288.23</v>
       </c>
       <c r="J7" t="n">
-        <v>300.79</v>
+        <v>296.14</v>
       </c>
       <c r="K7" t="n">
-        <v>313.06</v>
+        <v>312.39</v>
       </c>
       <c r="L7" t="n">
-        <v>325.42</v>
+        <v>324.75</v>
       </c>
       <c r="M7" t="n">
-        <v>337.9</v>
+        <v>337.23</v>
       </c>
       <c r="N7" t="n">
-        <v>350.48</v>
+        <v>349.81</v>
       </c>
       <c r="O7" t="n">
-        <v>363.17</v>
+        <v>362.5</v>
       </c>
       <c r="P7" t="n">
-        <v>375.97</v>
+        <v>375.3</v>
       </c>
       <c r="Q7" t="n">
-        <v>388.87</v>
+        <v>388.2</v>
       </c>
       <c r="R7" t="n">
-        <v>401.89</v>
+        <v>401.22</v>
       </c>
       <c r="S7" t="n">
-        <v>415</v>
+        <v>414.33</v>
       </c>
       <c r="T7" t="n">
-        <v>428.23</v>
+        <v>427.56</v>
       </c>
       <c r="U7" t="n">
-        <v>441.56</v>
+        <v>440.89</v>
       </c>
       <c r="V7" t="n">
-        <v>455</v>
+        <v>454.33</v>
       </c>
       <c r="W7" t="n">
-        <v>468.55</v>
+        <v>467.88</v>
       </c>
       <c r="X7" t="n">
-        <v>482.2</v>
+        <v>481.53</v>
       </c>
       <c r="Y7" t="n">
-        <v>495.96</v>
+        <v>495.29</v>
       </c>
       <c r="Z7" t="n">
-        <v>509.83</v>
+        <v>509.16</v>
       </c>
       <c r="AA7" t="n">
-        <v>523.8</v>
+        <v>523.13</v>
       </c>
       <c r="AB7" t="n">
-        <v>537.88</v>
+        <v>537.21</v>
       </c>
       <c r="AC7" t="n">
-        <v>552.0700000000001</v>
+        <v>551.4</v>
       </c>
       <c r="AD7" t="n">
-        <v>566.37</v>
+        <v>565.7</v>
       </c>
       <c r="AE7" t="n">
-        <v>580.77</v>
+        <v>580.1</v>
       </c>
       <c r="AF7" t="n">
-        <v>595.28</v>
+        <v>594.61</v>
       </c>
       <c r="AG7" t="n">
-        <v>609.9</v>
+        <v>609.23</v>
       </c>
       <c r="AH7" t="n">
-        <v>624.62</v>
+        <v>623.95</v>
       </c>
       <c r="AI7" t="n">
-        <v>639.45</v>
+        <v>638.78</v>
       </c>
       <c r="AJ7" t="n">
-        <v>654.39</v>
+        <v>653.72</v>
       </c>
     </row>
     <row r="8">
@@ -1482,88 +1482,88 @@
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>42.98</v>
+        <v>44.28</v>
       </c>
       <c r="J8" t="n">
-        <v>43.87</v>
+        <v>44.68</v>
       </c>
       <c r="K8" t="n">
-        <v>44.98</v>
+        <v>43.8</v>
       </c>
       <c r="L8" t="n">
-        <v>46.1</v>
+        <v>44.92</v>
       </c>
       <c r="M8" t="n">
-        <v>47.22</v>
+        <v>46.04</v>
       </c>
       <c r="N8" t="n">
-        <v>48.36</v>
+        <v>47.18</v>
       </c>
       <c r="O8" t="n">
-        <v>49.5</v>
+        <v>48.32</v>
       </c>
       <c r="P8" t="n">
-        <v>50.66</v>
+        <v>49.48</v>
       </c>
       <c r="Q8" t="n">
-        <v>51.82</v>
+        <v>50.64</v>
       </c>
       <c r="R8" t="n">
+        <v>51.81</v>
+      </c>
+      <c r="S8" t="n">
         <v>52.99</v>
       </c>
-      <c r="S8" t="n">
-        <v>54.17</v>
-      </c>
       <c r="T8" t="n">
-        <v>55.36</v>
+        <v>54.18</v>
       </c>
       <c r="U8" t="n">
-        <v>56.56</v>
+        <v>55.38</v>
       </c>
       <c r="V8" t="n">
-        <v>57.76</v>
+        <v>56.58</v>
       </c>
       <c r="W8" t="n">
-        <v>58.98</v>
+        <v>57.8</v>
       </c>
       <c r="X8" t="n">
-        <v>60.2</v>
+        <v>59.02</v>
       </c>
       <c r="Y8" t="n">
-        <v>61.44</v>
+        <v>60.26</v>
       </c>
       <c r="Z8" t="n">
-        <v>62.68</v>
+        <v>61.5</v>
       </c>
       <c r="AA8" t="n">
-        <v>63.93</v>
+        <v>62.75</v>
       </c>
       <c r="AB8" t="n">
-        <v>65.19</v>
+        <v>64.01000000000001</v>
       </c>
       <c r="AC8" t="n">
-        <v>66.45999999999999</v>
+        <v>65.28</v>
       </c>
       <c r="AD8" t="n">
-        <v>67.73999999999999</v>
+        <v>66.56</v>
       </c>
       <c r="AE8" t="n">
-        <v>69.02</v>
+        <v>67.84</v>
       </c>
       <c r="AF8" t="n">
-        <v>70.31999999999999</v>
+        <v>69.14</v>
       </c>
       <c r="AG8" t="n">
-        <v>71.62</v>
+        <v>70.44</v>
       </c>
       <c r="AH8" t="n">
-        <v>72.93000000000001</v>
+        <v>71.75</v>
       </c>
       <c r="AI8" t="n">
-        <v>74.26000000000001</v>
+        <v>73.08</v>
       </c>
       <c r="AJ8" t="n">
-        <v>75.59</v>
+        <v>74.41</v>
       </c>
     </row>
     <row r="9">
@@ -1730,88 +1730,88 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>127.3</v>
+        <v>129.57</v>
       </c>
       <c r="J10" t="n">
-        <v>133.11</v>
+        <v>137.75</v>
       </c>
       <c r="K10" t="n">
-        <v>139.61</v>
+        <v>140.3</v>
       </c>
       <c r="L10" t="n">
-        <v>146.17</v>
+        <v>146.86</v>
       </c>
       <c r="M10" t="n">
-        <v>152.78</v>
+        <v>153.47</v>
       </c>
       <c r="N10" t="n">
-        <v>159.46</v>
+        <v>160.15</v>
       </c>
       <c r="O10" t="n">
-        <v>166.19</v>
+        <v>166.88</v>
       </c>
       <c r="P10" t="n">
-        <v>172.98</v>
+        <v>173.67</v>
       </c>
       <c r="Q10" t="n">
-        <v>179.82</v>
+        <v>180.51</v>
       </c>
       <c r="R10" t="n">
-        <v>186.73</v>
+        <v>187.42</v>
       </c>
       <c r="S10" t="n">
-        <v>193.69</v>
+        <v>194.38</v>
       </c>
       <c r="T10" t="n">
-        <v>200.72</v>
+        <v>201.41</v>
       </c>
       <c r="U10" t="n">
-        <v>207.8</v>
+        <v>208.49</v>
       </c>
       <c r="V10" t="n">
-        <v>214.93</v>
+        <v>215.62</v>
       </c>
       <c r="W10" t="n">
-        <v>222.13</v>
+        <v>222.82</v>
       </c>
       <c r="X10" t="n">
-        <v>229.39</v>
+        <v>230.08</v>
       </c>
       <c r="Y10" t="n">
-        <v>236.7</v>
+        <v>237.39</v>
       </c>
       <c r="Z10" t="n">
-        <v>244.07</v>
+        <v>244.76</v>
       </c>
       <c r="AA10" t="n">
-        <v>251.5</v>
+        <v>252.19</v>
       </c>
       <c r="AB10" t="n">
-        <v>258.98</v>
+        <v>259.67</v>
       </c>
       <c r="AC10" t="n">
-        <v>266.53</v>
+        <v>267.22</v>
       </c>
       <c r="AD10" t="n">
-        <v>274.13</v>
+        <v>274.82</v>
       </c>
       <c r="AE10" t="n">
-        <v>281.79</v>
+        <v>282.48</v>
       </c>
       <c r="AF10" t="n">
-        <v>289.51</v>
+        <v>290.2</v>
       </c>
       <c r="AG10" t="n">
-        <v>297.29</v>
+        <v>297.98</v>
       </c>
       <c r="AH10" t="n">
-        <v>305.12</v>
+        <v>305.81</v>
       </c>
       <c r="AI10" t="n">
-        <v>313.01</v>
+        <v>313.7</v>
       </c>
       <c r="AJ10" t="n">
-        <v>320.96</v>
+        <v>321.65</v>
       </c>
     </row>
     <row r="11">
@@ -1854,88 +1854,88 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>44</v>
+        <v>47.17</v>
       </c>
       <c r="J11" t="n">
-        <v>45.53</v>
+        <v>48.54</v>
       </c>
       <c r="K11" t="n">
-        <v>47.3</v>
+        <v>48.77</v>
       </c>
       <c r="L11" t="n">
-        <v>49.08</v>
+        <v>50.55</v>
       </c>
       <c r="M11" t="n">
-        <v>50.88</v>
+        <v>52.35</v>
       </c>
       <c r="N11" t="n">
-        <v>52.69</v>
+        <v>54.16</v>
       </c>
       <c r="O11" t="n">
-        <v>54.52</v>
+        <v>55.99</v>
       </c>
       <c r="P11" t="n">
-        <v>56.36</v>
+        <v>57.83</v>
       </c>
       <c r="Q11" t="n">
-        <v>58.22</v>
+        <v>59.69</v>
       </c>
       <c r="R11" t="n">
-        <v>60.1</v>
+        <v>61.57</v>
       </c>
       <c r="S11" t="n">
-        <v>61.98</v>
+        <v>63.45</v>
       </c>
       <c r="T11" t="n">
-        <v>63.89</v>
+        <v>65.36</v>
       </c>
       <c r="U11" t="n">
-        <v>65.81</v>
+        <v>67.28</v>
       </c>
       <c r="V11" t="n">
-        <v>67.73999999999999</v>
+        <v>69.20999999999999</v>
       </c>
       <c r="W11" t="n">
-        <v>69.69</v>
+        <v>71.16</v>
       </c>
       <c r="X11" t="n">
-        <v>71.66</v>
+        <v>73.13</v>
       </c>
       <c r="Y11" t="n">
-        <v>73.64</v>
+        <v>75.11</v>
       </c>
       <c r="Z11" t="n">
-        <v>75.64</v>
+        <v>77.11</v>
       </c>
       <c r="AA11" t="n">
-        <v>77.65000000000001</v>
+        <v>79.12</v>
       </c>
       <c r="AB11" t="n">
-        <v>79.68000000000001</v>
+        <v>81.15000000000001</v>
       </c>
       <c r="AC11" t="n">
-        <v>81.72</v>
+        <v>83.19</v>
       </c>
       <c r="AD11" t="n">
-        <v>83.78</v>
+        <v>85.25</v>
       </c>
       <c r="AE11" t="n">
-        <v>85.84999999999999</v>
+        <v>87.31999999999999</v>
       </c>
       <c r="AF11" t="n">
-        <v>87.94</v>
+        <v>89.41</v>
       </c>
       <c r="AG11" t="n">
-        <v>90.04000000000001</v>
+        <v>91.51000000000001</v>
       </c>
       <c r="AH11" t="n">
-        <v>92.16</v>
+        <v>93.63</v>
       </c>
       <c r="AI11" t="n">
-        <v>94.29000000000001</v>
+        <v>95.76000000000001</v>
       </c>
       <c r="AJ11" t="n">
-        <v>96.44</v>
+        <v>97.91</v>
       </c>
     </row>
     <row r="12">
@@ -1978,88 +1978,88 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>42.64</v>
+        <v>43.14</v>
       </c>
       <c r="J12" t="n">
-        <v>43.94</v>
+        <v>44.46</v>
       </c>
       <c r="K12" t="n">
-        <v>45.47</v>
+        <v>46.16</v>
       </c>
       <c r="L12" t="n">
-        <v>47.02</v>
+        <v>47.71</v>
       </c>
       <c r="M12" t="n">
-        <v>48.57</v>
+        <v>49.26</v>
       </c>
       <c r="N12" t="n">
-        <v>50.14</v>
+        <v>50.83</v>
       </c>
       <c r="O12" t="n">
-        <v>51.73</v>
+        <v>52.42</v>
       </c>
       <c r="P12" t="n">
-        <v>53.32</v>
+        <v>54.01</v>
       </c>
       <c r="Q12" t="n">
-        <v>54.93</v>
+        <v>55.62</v>
       </c>
       <c r="R12" t="n">
-        <v>56.56</v>
+        <v>57.25</v>
       </c>
       <c r="S12" t="n">
-        <v>58.19</v>
+        <v>58.88</v>
       </c>
       <c r="T12" t="n">
-        <v>59.84</v>
+        <v>60.53</v>
       </c>
       <c r="U12" t="n">
-        <v>61.5</v>
+        <v>62.19</v>
       </c>
       <c r="V12" t="n">
-        <v>63.18</v>
+        <v>63.87</v>
       </c>
       <c r="W12" t="n">
-        <v>64.86</v>
+        <v>65.55</v>
       </c>
       <c r="X12" t="n">
-        <v>66.56</v>
+        <v>67.25</v>
       </c>
       <c r="Y12" t="n">
-        <v>68.28</v>
+        <v>68.97</v>
       </c>
       <c r="Z12" t="n">
-        <v>70</v>
+        <v>70.69</v>
       </c>
       <c r="AA12" t="n">
-        <v>71.73999999999999</v>
+        <v>72.43000000000001</v>
       </c>
       <c r="AB12" t="n">
-        <v>73.5</v>
+        <v>74.19</v>
       </c>
       <c r="AC12" t="n">
-        <v>75.26000000000001</v>
+        <v>75.95</v>
       </c>
       <c r="AD12" t="n">
-        <v>77.04000000000001</v>
+        <v>77.73</v>
       </c>
       <c r="AE12" t="n">
-        <v>78.83</v>
+        <v>79.52</v>
       </c>
       <c r="AF12" t="n">
-        <v>80.64</v>
+        <v>81.33</v>
       </c>
       <c r="AG12" t="n">
-        <v>82.45999999999999</v>
+        <v>83.15000000000001</v>
       </c>
       <c r="AH12" t="n">
-        <v>84.29000000000001</v>
+        <v>84.98</v>
       </c>
       <c r="AI12" t="n">
-        <v>86.13</v>
+        <v>86.81999999999999</v>
       </c>
       <c r="AJ12" t="n">
-        <v>87.98999999999999</v>
+        <v>88.68000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -2102,88 +2102,88 @@
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>1247.41</v>
+        <v>1241.42</v>
       </c>
       <c r="J13" t="n">
-        <v>1284.84</v>
+        <v>1279.49</v>
       </c>
       <c r="K13" t="n">
-        <v>1328.87</v>
+        <v>1324.32</v>
       </c>
       <c r="L13" t="n">
-        <v>1373.28</v>
+        <v>1368.73</v>
       </c>
       <c r="M13" t="n">
-        <v>1418.06</v>
+        <v>1413.51</v>
       </c>
       <c r="N13" t="n">
-        <v>1463.22</v>
+        <v>1458.67</v>
       </c>
       <c r="O13" t="n">
-        <v>1508.75</v>
+        <v>1504.2</v>
       </c>
       <c r="P13" t="n">
-        <v>1554.65</v>
+        <v>1550.1</v>
       </c>
       <c r="Q13" t="n">
-        <v>1600.93</v>
+        <v>1596.38</v>
       </c>
       <c r="R13" t="n">
-        <v>1647.58</v>
+        <v>1643.03</v>
       </c>
       <c r="S13" t="n">
-        <v>1694.61</v>
+        <v>1690.06</v>
       </c>
       <c r="T13" t="n">
-        <v>1742.01</v>
+        <v>1737.46</v>
       </c>
       <c r="U13" t="n">
-        <v>1789.79</v>
+        <v>1785.24</v>
       </c>
       <c r="V13" t="n">
-        <v>1837.94</v>
+        <v>1833.39</v>
       </c>
       <c r="W13" t="n">
-        <v>1886.46</v>
+        <v>1881.91</v>
       </c>
       <c r="X13" t="n">
-        <v>1935.36</v>
+        <v>1930.81</v>
       </c>
       <c r="Y13" t="n">
-        <v>1984.64</v>
+        <v>1980.09</v>
       </c>
       <c r="Z13" t="n">
-        <v>2034.28</v>
+        <v>2029.73</v>
       </c>
       <c r="AA13" t="n">
-        <v>2084.3</v>
+        <v>2079.75</v>
       </c>
       <c r="AB13" t="n">
-        <v>2134.7</v>
+        <v>2130.15</v>
       </c>
       <c r="AC13" t="n">
-        <v>2185.47</v>
+        <v>2180.92</v>
       </c>
       <c r="AD13" t="n">
-        <v>2236.61</v>
+        <v>2232.06</v>
       </c>
       <c r="AE13" t="n">
-        <v>2288.13</v>
+        <v>2283.58</v>
       </c>
       <c r="AF13" t="n">
-        <v>2340.02</v>
+        <v>2335.47</v>
       </c>
       <c r="AG13" t="n">
-        <v>2392.29</v>
+        <v>2387.74</v>
       </c>
       <c r="AH13" t="n">
-        <v>2444.93</v>
+        <v>2440.38</v>
       </c>
       <c r="AI13" t="n">
-        <v>2497.95</v>
+        <v>2493.4</v>
       </c>
       <c r="AJ13" t="n">
-        <v>2551.34</v>
+        <v>2546.79</v>
       </c>
     </row>
     <row r="14">
@@ -2226,88 +2226,88 @@
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>17.39</v>
+        <v>20.33</v>
       </c>
       <c r="J14" t="n">
-        <v>18.18</v>
+        <v>21.29</v>
       </c>
       <c r="K14" t="n">
-        <v>19.07</v>
+        <v>22.54</v>
       </c>
       <c r="L14" t="n">
-        <v>19.97</v>
+        <v>23.44</v>
       </c>
       <c r="M14" t="n">
-        <v>20.87</v>
+        <v>24.34</v>
       </c>
       <c r="N14" t="n">
-        <v>21.79</v>
+        <v>25.26</v>
       </c>
       <c r="O14" t="n">
-        <v>22.71</v>
+        <v>26.18</v>
       </c>
       <c r="P14" t="n">
-        <v>23.64</v>
+        <v>27.11</v>
       </c>
       <c r="Q14" t="n">
-        <v>24.57</v>
+        <v>28.04</v>
       </c>
       <c r="R14" t="n">
-        <v>25.52</v>
+        <v>28.99</v>
       </c>
       <c r="S14" t="n">
-        <v>26.47</v>
+        <v>29.94</v>
       </c>
       <c r="T14" t="n">
-        <v>27.43</v>
+        <v>30.9</v>
       </c>
       <c r="U14" t="n">
-        <v>28.4</v>
+        <v>31.87</v>
       </c>
       <c r="V14" t="n">
-        <v>29.38</v>
+        <v>32.85</v>
       </c>
       <c r="W14" t="n">
-        <v>30.36</v>
+        <v>33.83</v>
       </c>
       <c r="X14" t="n">
-        <v>31.36</v>
+        <v>34.83</v>
       </c>
       <c r="Y14" t="n">
-        <v>32.36</v>
+        <v>35.83</v>
       </c>
       <c r="Z14" t="n">
-        <v>33.37</v>
+        <v>36.84</v>
       </c>
       <c r="AA14" t="n">
-        <v>34.38</v>
+        <v>37.85</v>
       </c>
       <c r="AB14" t="n">
-        <v>35.41</v>
+        <v>38.88</v>
       </c>
       <c r="AC14" t="n">
-        <v>36.44</v>
+        <v>39.91</v>
       </c>
       <c r="AD14" t="n">
-        <v>37.48</v>
+        <v>40.95</v>
       </c>
       <c r="AE14" t="n">
-        <v>38.53</v>
+        <v>42</v>
       </c>
       <c r="AF14" t="n">
-        <v>39.58</v>
+        <v>43.05</v>
       </c>
       <c r="AG14" t="n">
-        <v>40.65</v>
+        <v>44.12</v>
       </c>
       <c r="AH14" t="n">
-        <v>41.72</v>
+        <v>45.19</v>
       </c>
       <c r="AI14" t="n">
-        <v>42.8</v>
+        <v>46.27</v>
       </c>
       <c r="AJ14" t="n">
-        <v>43.89</v>
+        <v>47.36</v>
       </c>
     </row>
     <row r="15">
@@ -2350,88 +2350,88 @@
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>52.31</v>
+        <v>51.79</v>
       </c>
       <c r="J15" t="n">
-        <v>54.86</v>
+        <v>52.92</v>
       </c>
       <c r="K15" t="n">
-        <v>57.7</v>
+        <v>56.46</v>
       </c>
       <c r="L15" t="n">
-        <v>60.56</v>
+        <v>59.32</v>
       </c>
       <c r="M15" t="n">
-        <v>63.44</v>
+        <v>62.2</v>
       </c>
       <c r="N15" t="n">
-        <v>66.34999999999999</v>
+        <v>65.11</v>
       </c>
       <c r="O15" t="n">
-        <v>69.29000000000001</v>
+        <v>68.05</v>
       </c>
       <c r="P15" t="n">
-        <v>72.25</v>
+        <v>71.01000000000001</v>
       </c>
       <c r="Q15" t="n">
-        <v>75.23999999999999</v>
+        <v>74</v>
       </c>
       <c r="R15" t="n">
-        <v>78.25</v>
+        <v>77.01000000000001</v>
       </c>
       <c r="S15" t="n">
-        <v>81.29000000000001</v>
+        <v>80.05</v>
       </c>
       <c r="T15" t="n">
-        <v>84.34999999999999</v>
+        <v>83.11</v>
       </c>
       <c r="U15" t="n">
-        <v>87.44</v>
+        <v>86.2</v>
       </c>
       <c r="V15" t="n">
-        <v>90.56</v>
+        <v>89.31999999999999</v>
       </c>
       <c r="W15" t="n">
-        <v>93.7</v>
+        <v>92.45999999999999</v>
       </c>
       <c r="X15" t="n">
-        <v>96.86</v>
+        <v>95.62</v>
       </c>
       <c r="Y15" t="n">
-        <v>100.06</v>
+        <v>98.81999999999999</v>
       </c>
       <c r="Z15" t="n">
-        <v>103.27</v>
+        <v>102.03</v>
       </c>
       <c r="AA15" t="n">
-        <v>106.52</v>
+        <v>105.28</v>
       </c>
       <c r="AB15" t="n">
-        <v>109.78</v>
+        <v>108.54</v>
       </c>
       <c r="AC15" t="n">
-        <v>113.08</v>
+        <v>111.84</v>
       </c>
       <c r="AD15" t="n">
-        <v>116.39</v>
+        <v>115.15</v>
       </c>
       <c r="AE15" t="n">
-        <v>119.74</v>
+        <v>118.5</v>
       </c>
       <c r="AF15" t="n">
-        <v>123.11</v>
+        <v>121.87</v>
       </c>
       <c r="AG15" t="n">
-        <v>126.5</v>
+        <v>125.26</v>
       </c>
       <c r="AH15" t="n">
-        <v>129.92</v>
+        <v>128.68</v>
       </c>
       <c r="AI15" t="n">
-        <v>133.37</v>
+        <v>132.13</v>
       </c>
       <c r="AJ15" t="n">
-        <v>136.84</v>
+        <v>135.6</v>
       </c>
     </row>
     <row r="16">
@@ -2474,88 +2474,88 @@
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>223.45</v>
+        <v>223.04</v>
       </c>
       <c r="J16" t="n">
         <v>233.01</v>
       </c>
       <c r="K16" t="n">
-        <v>243.79</v>
+        <v>243.77</v>
       </c>
       <c r="L16" t="n">
-        <v>254.66</v>
+        <v>254.64</v>
       </c>
       <c r="M16" t="n">
-        <v>265.63</v>
+        <v>265.61</v>
       </c>
       <c r="N16" t="n">
-        <v>276.69</v>
+        <v>276.67</v>
       </c>
       <c r="O16" t="n">
-        <v>287.85</v>
+        <v>287.83</v>
       </c>
       <c r="P16" t="n">
-        <v>299.11</v>
+        <v>299.09</v>
       </c>
       <c r="Q16" t="n">
-        <v>310.46</v>
+        <v>310.44</v>
       </c>
       <c r="R16" t="n">
-        <v>321.9</v>
+        <v>321.88</v>
       </c>
       <c r="S16" t="n">
-        <v>333.44</v>
+        <v>333.42</v>
       </c>
       <c r="T16" t="n">
-        <v>345.08</v>
+        <v>345.06</v>
       </c>
       <c r="U16" t="n">
-        <v>356.81</v>
+        <v>356.79</v>
       </c>
       <c r="V16" t="n">
-        <v>368.64</v>
+        <v>368.62</v>
       </c>
       <c r="W16" t="n">
-        <v>380.57</v>
+        <v>380.55</v>
       </c>
       <c r="X16" t="n">
-        <v>392.59</v>
+        <v>392.57</v>
       </c>
       <c r="Y16" t="n">
-        <v>404.7</v>
+        <v>404.68</v>
       </c>
       <c r="Z16" t="n">
-        <v>416.91</v>
+        <v>416.89</v>
       </c>
       <c r="AA16" t="n">
-        <v>429.22</v>
+        <v>429.2</v>
       </c>
       <c r="AB16" t="n">
-        <v>441.62</v>
+        <v>441.6</v>
       </c>
       <c r="AC16" t="n">
-        <v>454.12</v>
+        <v>454.1</v>
       </c>
       <c r="AD16" t="n">
-        <v>466.71</v>
+        <v>466.69</v>
       </c>
       <c r="AE16" t="n">
-        <v>479.4</v>
+        <v>479.38</v>
       </c>
       <c r="AF16" t="n">
-        <v>492.19</v>
+        <v>492.17</v>
       </c>
       <c r="AG16" t="n">
-        <v>505.07</v>
+        <v>505.05</v>
       </c>
       <c r="AH16" t="n">
-        <v>518.04</v>
+        <v>518.02</v>
       </c>
       <c r="AI16" t="n">
-        <v>531.12</v>
+        <v>531.1</v>
       </c>
       <c r="AJ16" t="n">
-        <v>544.28</v>
+        <v>544.26</v>
       </c>
     </row>
     <row r="17">
@@ -2598,88 +2598,88 @@
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>190.95</v>
+        <v>81.55</v>
       </c>
       <c r="J17" t="n">
-        <v>203.13</v>
+        <v>145.53</v>
       </c>
       <c r="K17" t="n">
-        <v>216.39</v>
+        <v>129.94</v>
       </c>
       <c r="L17" t="n">
-        <v>229.77</v>
+        <v>143.32</v>
       </c>
       <c r="M17" t="n">
-        <v>243.28</v>
+        <v>156.83</v>
       </c>
       <c r="N17" t="n">
-        <v>256.9</v>
+        <v>170.45</v>
       </c>
       <c r="O17" t="n">
-        <v>270.65</v>
+        <v>184.2</v>
       </c>
       <c r="P17" t="n">
-        <v>284.52</v>
+        <v>198.07</v>
       </c>
       <c r="Q17" t="n">
-        <v>298.51</v>
+        <v>212.06</v>
       </c>
       <c r="R17" t="n">
-        <v>312.62</v>
+        <v>226.17</v>
       </c>
       <c r="S17" t="n">
-        <v>326.85</v>
+        <v>240.4</v>
       </c>
       <c r="T17" t="n">
-        <v>341.21</v>
+        <v>254.76</v>
       </c>
       <c r="U17" t="n">
-        <v>355.68</v>
+        <v>269.23</v>
       </c>
       <c r="V17" t="n">
-        <v>370.28</v>
+        <v>283.83</v>
       </c>
       <c r="W17" t="n">
-        <v>385</v>
+        <v>298.55</v>
       </c>
       <c r="X17" t="n">
-        <v>399.85</v>
+        <v>313.4</v>
       </c>
       <c r="Y17" t="n">
-        <v>414.81</v>
+        <v>328.36</v>
       </c>
       <c r="Z17" t="n">
-        <v>429.9</v>
+        <v>343.45</v>
       </c>
       <c r="AA17" t="n">
-        <v>445.11</v>
+        <v>358.66</v>
       </c>
       <c r="AB17" t="n">
-        <v>460.44</v>
+        <v>373.99</v>
       </c>
       <c r="AC17" t="n">
-        <v>475.89</v>
+        <v>389.44</v>
       </c>
       <c r="AD17" t="n">
-        <v>491.46</v>
+        <v>405.01</v>
       </c>
       <c r="AE17" t="n">
-        <v>507.16</v>
+        <v>420.71</v>
       </c>
       <c r="AF17" t="n">
-        <v>522.98</v>
+        <v>436.53</v>
       </c>
       <c r="AG17" t="n">
-        <v>538.92</v>
+        <v>452.47</v>
       </c>
       <c r="AH17" t="n">
-        <v>554.98</v>
+        <v>468.53</v>
       </c>
       <c r="AI17" t="n">
-        <v>571.16</v>
+        <v>484.71</v>
       </c>
       <c r="AJ17" t="n">
-        <v>587.47</v>
+        <v>501.02</v>
       </c>
     </row>
     <row r="18">
@@ -2722,88 +2722,88 @@
         <v>0</v>
       </c>
       <c r="I18" t="n">
-        <v>29.35</v>
+        <v>27.94</v>
       </c>
       <c r="J18" t="n">
-        <v>30.02</v>
+        <v>29.86</v>
       </c>
       <c r="K18" t="n">
-        <v>30.86</v>
+        <v>32.2</v>
       </c>
       <c r="L18" t="n">
-        <v>31.69</v>
+        <v>33.03</v>
       </c>
       <c r="M18" t="n">
-        <v>32.54</v>
+        <v>33.88</v>
       </c>
       <c r="N18" t="n">
-        <v>33.39</v>
+        <v>34.73</v>
       </c>
       <c r="O18" t="n">
-        <v>34.25</v>
+        <v>35.59</v>
       </c>
       <c r="P18" t="n">
-        <v>35.11</v>
+        <v>36.45</v>
       </c>
       <c r="Q18" t="n">
-        <v>35.99</v>
+        <v>37.33</v>
       </c>
       <c r="R18" t="n">
-        <v>36.87</v>
+        <v>38.21</v>
       </c>
       <c r="S18" t="n">
-        <v>37.75</v>
+        <v>39.09</v>
       </c>
       <c r="T18" t="n">
-        <v>38.64</v>
+        <v>39.98</v>
       </c>
       <c r="U18" t="n">
-        <v>39.54</v>
+        <v>40.88</v>
       </c>
       <c r="V18" t="n">
-        <v>40.45</v>
+        <v>41.79</v>
       </c>
       <c r="W18" t="n">
-        <v>41.36</v>
+        <v>42.7</v>
       </c>
       <c r="X18" t="n">
-        <v>42.28</v>
+        <v>43.62</v>
       </c>
       <c r="Y18" t="n">
-        <v>43.21</v>
+        <v>44.55</v>
       </c>
       <c r="Z18" t="n">
-        <v>44.14</v>
+        <v>45.48</v>
       </c>
       <c r="AA18" t="n">
-        <v>45.08</v>
+        <v>46.42</v>
       </c>
       <c r="AB18" t="n">
-        <v>46.03</v>
+        <v>47.37</v>
       </c>
       <c r="AC18" t="n">
-        <v>46.98</v>
+        <v>48.32</v>
       </c>
       <c r="AD18" t="n">
-        <v>47.94</v>
+        <v>49.28</v>
       </c>
       <c r="AE18" t="n">
-        <v>48.91</v>
+        <v>50.25</v>
       </c>
       <c r="AF18" t="n">
-        <v>49.88</v>
+        <v>51.22</v>
       </c>
       <c r="AG18" t="n">
-        <v>50.86</v>
+        <v>52.2</v>
       </c>
       <c r="AH18" t="n">
-        <v>51.85</v>
+        <v>53.19</v>
       </c>
       <c r="AI18" t="n">
-        <v>52.84</v>
+        <v>54.18</v>
       </c>
       <c r="AJ18" t="n">
-        <v>53.84</v>
+        <v>55.18</v>
       </c>
     </row>
     <row r="19">
@@ -2846,88 +2846,88 @@
         <v>0</v>
       </c>
       <c r="I19" t="n">
-        <v>46.36</v>
+        <v>50.51</v>
       </c>
       <c r="J19" t="n">
-        <v>47.45</v>
+        <v>40.18</v>
       </c>
       <c r="K19" t="n">
-        <v>48.79</v>
+        <v>44.74</v>
       </c>
       <c r="L19" t="n">
-        <v>50.14</v>
+        <v>46.09</v>
       </c>
       <c r="M19" t="n">
-        <v>51.49</v>
+        <v>47.44</v>
       </c>
       <c r="N19" t="n">
-        <v>52.86</v>
+        <v>48.81</v>
       </c>
       <c r="O19" t="n">
-        <v>54.24</v>
+        <v>50.19</v>
       </c>
       <c r="P19" t="n">
-        <v>55.64</v>
+        <v>51.59</v>
       </c>
       <c r="Q19" t="n">
-        <v>57.04</v>
+        <v>52.99</v>
       </c>
       <c r="R19" t="n">
-        <v>58.45</v>
+        <v>54.4</v>
       </c>
       <c r="S19" t="n">
-        <v>59.88</v>
+        <v>55.83</v>
       </c>
       <c r="T19" t="n">
-        <v>61.31</v>
+        <v>57.26</v>
       </c>
       <c r="U19" t="n">
-        <v>62.76</v>
+        <v>58.71</v>
       </c>
       <c r="V19" t="n">
-        <v>64.20999999999999</v>
+        <v>60.16</v>
       </c>
       <c r="W19" t="n">
-        <v>65.68000000000001</v>
+        <v>61.63</v>
       </c>
       <c r="X19" t="n">
-        <v>67.16</v>
+        <v>63.11</v>
       </c>
       <c r="Y19" t="n">
-        <v>68.65000000000001</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="Z19" t="n">
-        <v>70.15000000000001</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="AA19" t="n">
-        <v>71.66</v>
+        <v>67.61</v>
       </c>
       <c r="AB19" t="n">
-        <v>73.19</v>
+        <v>69.14</v>
       </c>
       <c r="AC19" t="n">
-        <v>74.72</v>
+        <v>70.67</v>
       </c>
       <c r="AD19" t="n">
-        <v>76.27</v>
+        <v>72.22</v>
       </c>
       <c r="AE19" t="n">
-        <v>77.81999999999999</v>
+        <v>73.77</v>
       </c>
       <c r="AF19" t="n">
-        <v>79.39</v>
+        <v>75.34</v>
       </c>
       <c r="AG19" t="n">
-        <v>80.95999999999999</v>
+        <v>76.91</v>
       </c>
       <c r="AH19" t="n">
-        <v>82.55</v>
+        <v>78.5</v>
       </c>
       <c r="AI19" t="n">
-        <v>84.15000000000001</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="AJ19" t="n">
-        <v>85.76000000000001</v>
+        <v>81.70999999999999</v>
       </c>
     </row>
     <row r="20">

</xml_diff>